<commit_message>
Preview physical escape-room puzzles and resumable object discoveries
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template-v2.xlsx
+++ b/public/labs/first-love/first-love-template-v2.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R22b9e12509674b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R63e3bbe383b54636"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R9d80f61a460b47a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="Re2b031147fb945b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R01e8f8af0bc64b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R7d09c5d3684948c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R787a80c5b7f84cba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R89fc82289746473e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R2a6ffed87857400b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R850c8141c1a24ff4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R89a655620881454d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R85156d09d43641f9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -473,7 +473,7 @@
         <x:v>오늘은 미루지 않기로 했다</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>각자 가진 정보를 모아 네 메모를 분류하세요.</x:v>
+        <x:v>메모를 알맞은 주머니에 넣어 파일을 여세요.</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
         <x:v>낱말을 품사에 따라 분류합니다.</x:v>
@@ -485,13 +485,13 @@
 라: 웃다 → 동사</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>각 메모에 적힌 정보를 담당 친구에게 물어보세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>같은 분류함에 여러 메모가 들어갈 수 있어요.</x:v>
+        <x:v>기록에 나온 정보를 분류 기준과 대조하세요.</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
-        <x:v>메모를 누른 뒤 분류함을 누르세요.</x:v>
+        <x:v>메모를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="78.75" customHeight="1">
@@ -508,22 +508,22 @@
         <x:v>같이 보던 책</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>네 관찰과 모두 맞는 기록 한 장을 고르세요.</x:v>
+        <x:v>관찰 기록과 맞는 책을 찾아 꺼내세요.</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
         <x:v>친구에게 서로 다른 관찰 결과를 물어보세요.</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>기록 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 기록도 남습니다.</x:v>
+        <x:v>책 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 책도 남습니다.</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>색·모양·줄 수·재질의 관찰을 모으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
-        <x:v>조건이 다른 기록을 하나씩 비교하세요.</x:v>
+        <x:v>네 관찰에 모두 맞는 물건인지 비교하세요.</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>마지막 기록을 누르고 정답 확인을 누르세요.</x:v>
+        <x:v>물건을 선택한 뒤 아래 손잡이 버튼을 누르세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="78.75" customHeight="1">
@@ -540,7 +540,7 @@
         <x:v>비밀 유지가 너무 철저한데</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>네 전달 메모를 모아 봉투를 순서대로 놓으세요.</x:v>
+        <x:v>봉투를 순서대로 끼워 서랍을 여세요.</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
         <x:v>메모의 앞·뒤는 왼쪽에서 오른쪽 순서입니다.</x:v>
@@ -549,13 +549,13 @@
         <x:v>나 → 라 → 가 → 다. 네 조건 중 하나라도 빼면 순서가 둘 이상 가능합니다.</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
-        <x:v>네 사람이 받은 전달 메모를 하나씩 읽으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>앞뒤 관계와 붙어 있는지를 함께 확인하세요.</x:v>
+        <x:v>앞뒤 관계와 이웃한 자리를 함께 확인하세요.</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>봉투를 누른 뒤 놓을 순서 칸을 누르세요.</x:v>
+        <x:v>봉투를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="78.75" customHeight="1">
@@ -572,7 +572,7 @@
         <x:v>수정본을 믿으면 안 되는 이유</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>각자 가진 정보를 모아 네 메모를 분류하세요.</x:v>
+        <x:v>기록표를 맞는 칸에 놓고 확인 도장을 누르세요.</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
         <x:v>0보다 크면 양수, 작으면 음수입니다.</x:v>
@@ -584,13 +584,13 @@
 라: +2 → 양수</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>각 메모에 적힌 정보를 담당 친구에게 물어보세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>같은 분류함에 여러 메모가 들어갈 수 있어요.</x:v>
+        <x:v>기록에 나온 정보를 분류 기준과 대조하세요.</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>메모를 누른 뒤 분류함을 누르세요.</x:v>
+        <x:v>기록표를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="78.75" customHeight="1">
@@ -607,22 +607,22 @@
         <x:v>내 것은 어느 쪽으로 갔는데</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>네 관찰과 모두 맞는 기록 한 장을 고르세요.</x:v>
+        <x:v>네 기록과 맞는 반납함의 걸쇠를 여세요.</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
         <x:v>친구에게 서로 다른 관찰 결과를 물어보세요.</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>기록 다만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 기록도 남습니다.</x:v>
+        <x:v>반납함 다만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 반납함도 남습니다.</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
-        <x:v>색·모양·줄 수·재질의 관찰을 모으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:v>조건이 다른 기록을 하나씩 비교하세요.</x:v>
+        <x:v>네 관찰에 모두 맞는 물건인지 비교하세요.</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
-        <x:v>마지막 기록을 누르고 정답 확인을 누르세요.</x:v>
+        <x:v>물건을 선택한 뒤 아래 손잡이 버튼을 누르세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="78.75" customHeight="1">
@@ -639,7 +639,7 @@
         <x:v>확성기는 왜 있는데</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>네 전달 메모를 모아 봉투를 순서대로 놓으세요.</x:v>
+        <x:v>연결표를 순서대로 꽂고 레버를 내리세요.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
         <x:v>메모의 앞·뒤는 왼쪽에서 오른쪽 순서입니다.</x:v>
@@ -648,13 +648,13 @@
         <x:v>나 → 라 → 가 → 다. 네 조건 중 하나라도 빼면 순서가 둘 이상 가능합니다.</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>네 사람이 받은 전달 메모를 하나씩 읽으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:v>앞뒤 관계와 붙어 있는지를 함께 확인하세요.</x:v>
+        <x:v>앞뒤 관계와 이웃한 자리를 함께 확인하세요.</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>봉투를 누른 뒤 놓을 순서 칸을 누르세요.</x:v>
+        <x:v>연결표를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="78.75" customHeight="1">
@@ -671,7 +671,7 @@
         <x:v>그냥 넣으면 안 되는 거야?</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>각자 가진 정보를 모아 네 메모를 분류하세요.</x:v>
+        <x:v>상자를 맞는 칸에 넣어 보관함을 여세요.</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
         <x:v>관찰한 생물을 동물과 식물로 분류합니다.</x:v>
@@ -683,13 +683,13 @@
 라: 강아지 → 동물</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>각 메모에 적힌 정보를 담당 친구에게 물어보세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>같은 분류함에 여러 메모가 들어갈 수 있어요.</x:v>
+        <x:v>기록에 나온 정보를 분류 기준과 대조하세요.</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>메모를 누른 뒤 분류함을 누르세요.</x:v>
+        <x:v>상자를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="78.75" customHeight="1">
@@ -706,22 +706,22 @@
         <x:v>이제 네가 가면 돼</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>네 관찰과 모두 맞는 기록 한 장을 고르세요.</x:v>
+        <x:v>네 기록과 맞는 봉투를 찾아 인수함을 여세요.</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
         <x:v>친구에게 서로 다른 관찰 결과를 물어보세요.</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
-        <x:v>기록 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 기록도 남습니다.</x:v>
+        <x:v>인수 봉투 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 인수 봉투도 남습니다.</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
-        <x:v>색·모양·줄 수·재질의 관찰을 모으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>조건이 다른 기록을 하나씩 비교하세요.</x:v>
+        <x:v>네 관찰에 모두 맞는 물건인지 비교하세요.</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>마지막 기록을 누르고 정답 확인을 누르세요.</x:v>
+        <x:v>물건을 선택한 뒤 아래 손잡이 버튼을 누르세요.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -899,7 +899,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>기록 가</x:v>
+        <x:v>책 가</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>빨강 · 원 · 두 줄 · 종이</x:v>
@@ -924,7 +924,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>기록 나</x:v>
+        <x:v>책 나</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>파랑 · 세모 · 두 줄 · 종이</x:v>
@@ -949,7 +949,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>기록 다</x:v>
+        <x:v>책 다</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
         <x:v>파랑 · 원 · 네 줄 · 종이</x:v>
@@ -974,7 +974,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>기록 라</x:v>
+        <x:v>책 라</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>파랑 · 원 · 두 줄 · 금속</x:v>
@@ -999,7 +999,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>기록 마</x:v>
+        <x:v>책 마</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>빨강 · 세모 · 네 줄 · 금속</x:v>
@@ -1024,7 +1024,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>기록 바</x:v>
+        <x:v>책 바</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
         <x:v>파랑 · 원 · 두 줄 · 종이</x:v>
@@ -1141,7 +1141,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>메모 가</x:v>
+        <x:v>기록표 가</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1166,7 +1166,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>메모 나</x:v>
+        <x:v>기록표 나</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1191,7 +1191,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>메모 다</x:v>
+        <x:v>기록표 다</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1216,7 +1216,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>메모 라</x:v>
+        <x:v>기록표 라</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1241,7 +1241,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>기록 가</x:v>
+        <x:v>반납함 가</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
         <x:v>노랑 · 별 · 한 줄 · 금속</x:v>
@@ -1266,7 +1266,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>기록 나</x:v>
+        <x:v>반납함 나</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
         <x:v>빨강 · 세모 · 네 줄 · 금속</x:v>
@@ -1291,7 +1291,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>기록 다</x:v>
+        <x:v>반납함 다</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
         <x:v>노랑 · 별 · 한 줄 · 천</x:v>
@@ -1316,7 +1316,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>기록 라</x:v>
+        <x:v>반납함 라</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
         <x:v>빨강 · 별 · 한 줄 · 천</x:v>
@@ -1341,7 +1341,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>기록 마</x:v>
+        <x:v>반납함 마</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
         <x:v>노랑 · 세모 · 한 줄 · 천</x:v>
@@ -1366,7 +1366,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>기록 바</x:v>
+        <x:v>반납함 바</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
         <x:v>노랑 · 별 · 네 줄 · 천</x:v>
@@ -1391,7 +1391,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>봉투 가</x:v>
+        <x:v>연결표 가</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str"/>
       <x:c r="E29" s="4" t="n">
@@ -1414,7 +1414,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>봉투 나</x:v>
+        <x:v>연결표 나</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str"/>
       <x:c r="E30" s="4" t="n">
@@ -1437,7 +1437,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>봉투 다</x:v>
+        <x:v>연결표 다</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str"/>
       <x:c r="E31" s="4" t="n">
@@ -1460,7 +1460,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>봉투 라</x:v>
+        <x:v>연결표 라</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str"/>
       <x:c r="E32" s="4" t="n">
@@ -1483,7 +1483,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>메모 가</x:v>
+        <x:v>상자 가</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1508,7 +1508,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>메모 나</x:v>
+        <x:v>상자 나</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1533,7 +1533,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>메모 다</x:v>
+        <x:v>상자 다</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1558,7 +1558,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>메모 라</x:v>
+        <x:v>상자 라</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
         <x:v>담당자의 단서와 연결</x:v>
@@ -1583,7 +1583,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>기록 가</x:v>
+        <x:v>인수 봉투 가</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
         <x:v>빨강 · 네모 · 세 줄 · 나무</x:v>
@@ -1608,7 +1608,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>기록 나</x:v>
+        <x:v>인수 봉투 나</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
         <x:v>초록 · 세모 · 세 줄 · 나무</x:v>
@@ -1633,7 +1633,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C39" s="9" t="str">
-        <x:v>기록 다</x:v>
+        <x:v>인수 봉투 다</x:v>
       </x:c>
       <x:c r="D39" s="9" t="str">
         <x:v>초록 · 네모 · 네 줄 · 나무</x:v>
@@ -1658,7 +1658,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
-        <x:v>기록 라</x:v>
+        <x:v>인수 봉투 라</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
         <x:v>초록 · 네모 · 세 줄 · 금속</x:v>
@@ -1683,7 +1683,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C41" s="9" t="str">
-        <x:v>기록 마</x:v>
+        <x:v>인수 봉투 마</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
         <x:v>빨강 · 세모 · 네 줄 · 금속</x:v>
@@ -1708,7 +1708,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>기록 바</x:v>
+        <x:v>인수 봉투 바</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
         <x:v>초록 · 네모 · 세 줄 · 나무</x:v>
@@ -1974,7 +1974,7 @@
         <x:v>색 관찰</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>내 사진에서 확인한 색: 파랑</x:v>
+        <x:v>내 관찰 책의 색: 파랑</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>B|C|D|F</x:v>
@@ -1991,7 +1991,7 @@
         <x:v>모양 관찰</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>내 사진에서 확인한 모양: 원</x:v>
+        <x:v>내 관찰 책의 모양: 원</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>A|C|D|F</x:v>
@@ -2008,7 +2008,7 @@
         <x:v>줄 관찰</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>내 사진에서 확인한 줄 수: 두 줄</x:v>
+        <x:v>내 관찰 책의 줄 수: 두 줄</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
         <x:v>A|B|D|F</x:v>
@@ -2025,7 +2025,7 @@
         <x:v>재질 관찰</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>내 사진에서 확인한 재질: 종이</x:v>
+        <x:v>내 관찰 책의 재질: 종이</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
         <x:v>A|B|C|F</x:v>
@@ -2107,10 +2107,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>메모 가의 정보</x:v>
+        <x:v>기록표 가의 정보</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>메모 가에 적힌 수: −3</x:v>
+        <x:v>기록표 가에 적힌 수: −3</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
         <x:v>A=T2</x:v>
@@ -2124,10 +2124,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>메모 나의 정보</x:v>
+        <x:v>기록표 나의 정보</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>메모 나에 적힌 수: +7</x:v>
+        <x:v>기록표 나에 적힌 수: +7</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
         <x:v>B=T1</x:v>
@@ -2141,10 +2141,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>메모 다의 정보</x:v>
+        <x:v>기록표 다의 정보</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>메모 다에 적힌 수: −8</x:v>
+        <x:v>기록표 다에 적힌 수: −8</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
         <x:v>C=T2</x:v>
@@ -2158,10 +2158,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>메모 라의 정보</x:v>
+        <x:v>기록표 라의 정보</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>메모 라에 적힌 수: +2</x:v>
+        <x:v>기록표 라에 적힌 수: +2</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
         <x:v>D=T1</x:v>
@@ -2178,7 +2178,7 @@
         <x:v>색 관찰</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>내 사진에서 확인한 색: 노랑</x:v>
+        <x:v>내 관찰 반납함의 색: 노랑</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
         <x:v>A|C|E|F</x:v>
@@ -2195,7 +2195,7 @@
         <x:v>모양 관찰</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>내 사진에서 확인한 모양: 별</x:v>
+        <x:v>내 관찰 반납함의 모양: 별</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
         <x:v>A|C|D|F</x:v>
@@ -2212,7 +2212,7 @@
         <x:v>줄 관찰</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>내 사진에서 확인한 줄 수: 한 줄</x:v>
+        <x:v>내 관찰 반납함의 줄 수: 한 줄</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
         <x:v>A|C|D|E</x:v>
@@ -2229,7 +2229,7 @@
         <x:v>재질 관찰</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>내 사진에서 확인한 재질: 천</x:v>
+        <x:v>내 관찰 반납함의 재질: 천</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
         <x:v>C|D|E|F</x:v>
@@ -2246,7 +2246,7 @@
         <x:v>앞뒤 메모</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>가 봉투는 나 봉투보다 뒤에 놓는다.</x:v>
+        <x:v>가 연결표는 나 연결표보다 뒤에 놓는다.</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
         <x:v>A&gt;B</x:v>
@@ -2263,7 +2263,7 @@
         <x:v>간격 메모</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>가 봉투와 나 봉투는 붙여 놓지 않는다.</x:v>
+        <x:v>가 연결표와 나 연결표는 붙여 놓지 않는다.</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
         <x:v>A!~B</x:v>
@@ -2280,7 +2280,7 @@
         <x:v>전달 메모</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>가 봉투는 라 봉투보다 뒤에 놓는다.</x:v>
+        <x:v>가 연결표는 라 연결표보다 뒤에 놓는다.</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
         <x:v>A&gt;D</x:v>
@@ -2297,7 +2297,7 @@
         <x:v>끝자리 메모</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>가 봉투는 마지막에 놓지 않는다.</x:v>
+        <x:v>가 연결표는 마지막에 놓지 않는다.</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
         <x:v>A!=4</x:v>
@@ -2311,10 +2311,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>메모 가의 정보</x:v>
+        <x:v>상자 가의 정보</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>메모 가에 적힌 생물: 고양이</x:v>
+        <x:v>상자 가에 적힌 생물: 고양이</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
         <x:v>A=T1</x:v>
@@ -2328,10 +2328,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>메모 나의 정보</x:v>
+        <x:v>상자 나의 정보</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>메모 나에 적힌 생물: 장미</x:v>
+        <x:v>상자 나에 적힌 생물: 장미</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
         <x:v>B=T2</x:v>
@@ -2345,10 +2345,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>메모 다의 정보</x:v>
+        <x:v>상자 다의 정보</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>메모 다에 적힌 생물: 민들레</x:v>
+        <x:v>상자 다에 적힌 생물: 민들레</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
         <x:v>C=T2</x:v>
@@ -2362,10 +2362,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>메모 라의 정보</x:v>
+        <x:v>상자 라의 정보</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>메모 라에 적힌 생물: 강아지</x:v>
+        <x:v>상자 라에 적힌 생물: 강아지</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
         <x:v>D=T1</x:v>
@@ -2382,7 +2382,7 @@
         <x:v>색 관찰</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>내 사진에서 확인한 색: 초록</x:v>
+        <x:v>내 관찰 인수 봉투의 색: 초록</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
         <x:v>B|C|D|F</x:v>
@@ -2399,7 +2399,7 @@
         <x:v>모양 관찰</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>내 사진에서 확인한 모양: 네모</x:v>
+        <x:v>내 관찰 인수 봉투의 모양: 네모</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
         <x:v>A|C|D|F</x:v>
@@ -2416,7 +2416,7 @@
         <x:v>줄 관찰</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>내 사진에서 확인한 줄 수: 세 줄</x:v>
+        <x:v>내 관찰 인수 봉투의 줄 수: 세 줄</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
         <x:v>A|B|D|F</x:v>
@@ -2433,7 +2433,7 @@
         <x:v>재질 관찰</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
-        <x:v>내 사진에서 확인한 재질: 나무</x:v>
+        <x:v>내 관찰 인수 봉투의 재질: 나무</x:v>
       </x:c>
       <x:c r="E36" s="9" t="str">
         <x:v>A|B|C|F</x:v>

</xml_diff>

<commit_message>
Fit physical puzzle objects to compact screens and shape the return bookshelf
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template-v2.xlsx
+++ b/public/labs/first-love/first-love-template-v2.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R787a80c5b7f84cba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R89fc82289746473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R2a6ffed87857400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R850c8141c1a24ff4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R89a655620881454d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R85156d09d43641f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="Rc983cc98972849be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="Re60799e8242e48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R722ac35335874502"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R99b18ac83d834ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R127dc3f809c74fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R94fb811c9b154ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -801,9 +801,7 @@
       <x:c r="C5" s="9" t="str">
         <x:v>메모 가</x:v>
       </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D5" s="9" t="str"/>
       <x:c r="E5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -826,9 +824,7 @@
       <x:c r="C6" s="9" t="str">
         <x:v>메모 나</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D6" s="9" t="str"/>
       <x:c r="E6" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -851,9 +847,7 @@
       <x:c r="C7" s="9" t="str">
         <x:v>메모 다</x:v>
       </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D7" s="9" t="str"/>
       <x:c r="E7" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -876,9 +870,7 @@
       <x:c r="C8" s="9" t="str">
         <x:v>메모 라</x:v>
       </x:c>
-      <x:c r="D8" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D8" s="9" t="str"/>
       <x:c r="E8" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1143,9 +1135,7 @@
       <x:c r="C19" s="9" t="str">
         <x:v>기록표 가</x:v>
       </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D19" s="9" t="str"/>
       <x:c r="E19" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1168,9 +1158,7 @@
       <x:c r="C20" s="9" t="str">
         <x:v>기록표 나</x:v>
       </x:c>
-      <x:c r="D20" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D20" s="9" t="str"/>
       <x:c r="E20" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1193,9 +1181,7 @@
       <x:c r="C21" s="9" t="str">
         <x:v>기록표 다</x:v>
       </x:c>
-      <x:c r="D21" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D21" s="9" t="str"/>
       <x:c r="E21" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1218,9 +1204,7 @@
       <x:c r="C22" s="9" t="str">
         <x:v>기록표 라</x:v>
       </x:c>
-      <x:c r="D22" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D22" s="9" t="str"/>
       <x:c r="E22" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1485,9 +1469,7 @@
       <x:c r="C33" s="9" t="str">
         <x:v>상자 가</x:v>
       </x:c>
-      <x:c r="D33" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D33" s="9" t="str"/>
       <x:c r="E33" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1510,9 +1492,7 @@
       <x:c r="C34" s="9" t="str">
         <x:v>상자 나</x:v>
       </x:c>
-      <x:c r="D34" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D34" s="9" t="str"/>
       <x:c r="E34" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1535,9 +1515,7 @@
       <x:c r="C35" s="9" t="str">
         <x:v>상자 다</x:v>
       </x:c>
-      <x:c r="D35" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D35" s="9" t="str"/>
       <x:c r="E35" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1560,9 +1538,7 @@
       <x:c r="C36" s="9" t="str">
         <x:v>상자 라</x:v>
       </x:c>
-      <x:c r="D36" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D36" s="9" t="str"/>
       <x:c r="E36" s="4" t="n">
         <x:v>0</x:v>
       </x:c>

</xml_diff>

<commit_message>
Turn first-love cooperative puzzles into physical escape-room devices
Add role-private clue discoveries, interactive books, envelopes, drawers and sockets, and resumable object reveals before story transitions. Preserve subject-independent validation and legacy lessons. Update workbook and authoring guidance; verify 30 tests and responsive device flows.
</commit_message>
<xml_diff>
--- a/public/labs/first-love/first-love-template-v2.xlsx
+++ b/public/labs/first-love/first-love-template-v2.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R22b9e12509674b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="R63e3bbe383b54636"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R9d80f61a460b47a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="Re2b031147fb945b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R01e8f8af0bc64b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R7d09c5d3684948c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="Rc983cc98972849be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="퍼즐" sheetId="2" r:id="Re60799e8242e48fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="자료" sheetId="3" r:id="R722ac35335874502"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="대상" sheetId="4" r:id="R99b18ac83d834ad4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모둠단서" sheetId="5" r:id="R127dc3f809c74fae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="장치" sheetId="6" r:id="R94fb811c9b154ed3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -473,7 +473,7 @@
         <x:v>오늘은 미루지 않기로 했다</x:v>
       </x:c>
       <x:c r="E5" s="9" t="str">
-        <x:v>각자 가진 정보를 모아 네 메모를 분류하세요.</x:v>
+        <x:v>메모를 알맞은 주머니에 넣어 파일을 여세요.</x:v>
       </x:c>
       <x:c r="F5" s="9" t="str">
         <x:v>낱말을 품사에 따라 분류합니다.</x:v>
@@ -485,13 +485,13 @@
 라: 웃다 → 동사</x:v>
       </x:c>
       <x:c r="H5" s="9" t="str">
-        <x:v>각 메모에 적힌 정보를 담당 친구에게 물어보세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I5" s="9" t="str">
-        <x:v>같은 분류함에 여러 메모가 들어갈 수 있어요.</x:v>
+        <x:v>기록에 나온 정보를 분류 기준과 대조하세요.</x:v>
       </x:c>
       <x:c r="J5" s="9" t="str">
-        <x:v>메모를 누른 뒤 분류함을 누르세요.</x:v>
+        <x:v>메모를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="78.75" customHeight="1">
@@ -508,22 +508,22 @@
         <x:v>같이 보던 책</x:v>
       </x:c>
       <x:c r="E6" s="9" t="str">
-        <x:v>네 관찰과 모두 맞는 기록 한 장을 고르세요.</x:v>
+        <x:v>관찰 기록과 맞는 책을 찾아 꺼내세요.</x:v>
       </x:c>
       <x:c r="F6" s="9" t="str">
         <x:v>친구에게 서로 다른 관찰 결과를 물어보세요.</x:v>
       </x:c>
       <x:c r="G6" s="9" t="str">
-        <x:v>기록 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 기록도 남습니다.</x:v>
+        <x:v>책 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 책도 남습니다.</x:v>
       </x:c>
       <x:c r="H6" s="9" t="str">
-        <x:v>색·모양·줄 수·재질의 관찰을 모으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I6" s="9" t="str">
-        <x:v>조건이 다른 기록을 하나씩 비교하세요.</x:v>
+        <x:v>네 관찰에 모두 맞는 물건인지 비교하세요.</x:v>
       </x:c>
       <x:c r="J6" s="9" t="str">
-        <x:v>마지막 기록을 누르고 정답 확인을 누르세요.</x:v>
+        <x:v>물건을 선택한 뒤 아래 손잡이 버튼을 누르세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="78.75" customHeight="1">
@@ -540,7 +540,7 @@
         <x:v>비밀 유지가 너무 철저한데</x:v>
       </x:c>
       <x:c r="E7" s="9" t="str">
-        <x:v>네 전달 메모를 모아 봉투를 순서대로 놓으세요.</x:v>
+        <x:v>봉투를 순서대로 끼워 서랍을 여세요.</x:v>
       </x:c>
       <x:c r="F7" s="9" t="str">
         <x:v>메모의 앞·뒤는 왼쪽에서 오른쪽 순서입니다.</x:v>
@@ -549,13 +549,13 @@
         <x:v>나 → 라 → 가 → 다. 네 조건 중 하나라도 빼면 순서가 둘 이상 가능합니다.</x:v>
       </x:c>
       <x:c r="H7" s="9" t="str">
-        <x:v>네 사람이 받은 전달 메모를 하나씩 읽으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I7" s="9" t="str">
-        <x:v>앞뒤 관계와 붙어 있는지를 함께 확인하세요.</x:v>
+        <x:v>앞뒤 관계와 이웃한 자리를 함께 확인하세요.</x:v>
       </x:c>
       <x:c r="J7" s="9" t="str">
-        <x:v>봉투를 누른 뒤 놓을 순서 칸을 누르세요.</x:v>
+        <x:v>봉투를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="78.75" customHeight="1">
@@ -572,7 +572,7 @@
         <x:v>수정본을 믿으면 안 되는 이유</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>각자 가진 정보를 모아 네 메모를 분류하세요.</x:v>
+        <x:v>기록표를 맞는 칸에 놓고 확인 도장을 누르세요.</x:v>
       </x:c>
       <x:c r="F8" s="9" t="str">
         <x:v>0보다 크면 양수, 작으면 음수입니다.</x:v>
@@ -584,13 +584,13 @@
 라: +2 → 양수</x:v>
       </x:c>
       <x:c r="H8" s="9" t="str">
-        <x:v>각 메모에 적힌 정보를 담당 친구에게 물어보세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I8" s="9" t="str">
-        <x:v>같은 분류함에 여러 메모가 들어갈 수 있어요.</x:v>
+        <x:v>기록에 나온 정보를 분류 기준과 대조하세요.</x:v>
       </x:c>
       <x:c r="J8" s="9" t="str">
-        <x:v>메모를 누른 뒤 분류함을 누르세요.</x:v>
+        <x:v>기록표를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="78.75" customHeight="1">
@@ -607,22 +607,22 @@
         <x:v>내 것은 어느 쪽으로 갔는데</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>네 관찰과 모두 맞는 기록 한 장을 고르세요.</x:v>
+        <x:v>네 기록과 맞는 반납함의 걸쇠를 여세요.</x:v>
       </x:c>
       <x:c r="F9" s="9" t="str">
         <x:v>친구에게 서로 다른 관찰 결과를 물어보세요.</x:v>
       </x:c>
       <x:c r="G9" s="9" t="str">
-        <x:v>기록 다만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 기록도 남습니다.</x:v>
+        <x:v>반납함 다만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 반납함도 남습니다.</x:v>
       </x:c>
       <x:c r="H9" s="9" t="str">
-        <x:v>색·모양·줄 수·재질의 관찰을 모으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I9" s="9" t="str">
-        <x:v>조건이 다른 기록을 하나씩 비교하세요.</x:v>
+        <x:v>네 관찰에 모두 맞는 물건인지 비교하세요.</x:v>
       </x:c>
       <x:c r="J9" s="9" t="str">
-        <x:v>마지막 기록을 누르고 정답 확인을 누르세요.</x:v>
+        <x:v>물건을 선택한 뒤 아래 손잡이 버튼을 누르세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="78.75" customHeight="1">
@@ -639,7 +639,7 @@
         <x:v>확성기는 왜 있는데</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>네 전달 메모를 모아 봉투를 순서대로 놓으세요.</x:v>
+        <x:v>연결표를 순서대로 꽂고 레버를 내리세요.</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
         <x:v>메모의 앞·뒤는 왼쪽에서 오른쪽 순서입니다.</x:v>
@@ -648,13 +648,13 @@
         <x:v>나 → 라 → 가 → 다. 네 조건 중 하나라도 빼면 순서가 둘 이상 가능합니다.</x:v>
       </x:c>
       <x:c r="H10" s="9" t="str">
-        <x:v>네 사람이 받은 전달 메모를 하나씩 읽으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I10" s="9" t="str">
-        <x:v>앞뒤 관계와 붙어 있는지를 함께 확인하세요.</x:v>
+        <x:v>앞뒤 관계와 이웃한 자리를 함께 확인하세요.</x:v>
       </x:c>
       <x:c r="J10" s="9" t="str">
-        <x:v>봉투를 누른 뒤 놓을 순서 칸을 누르세요.</x:v>
+        <x:v>연결표를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="78.75" customHeight="1">
@@ -671,7 +671,7 @@
         <x:v>그냥 넣으면 안 되는 거야?</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>각자 가진 정보를 모아 네 메모를 분류하세요.</x:v>
+        <x:v>상자를 맞는 칸에 넣어 보관함을 여세요.</x:v>
       </x:c>
       <x:c r="F11" s="9" t="str">
         <x:v>관찰한 생물을 동물과 식물로 분류합니다.</x:v>
@@ -683,13 +683,13 @@
 라: 강아지 → 동물</x:v>
       </x:c>
       <x:c r="H11" s="9" t="str">
-        <x:v>각 메모에 적힌 정보를 담당 친구에게 물어보세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I11" s="9" t="str">
-        <x:v>같은 분류함에 여러 메모가 들어갈 수 있어요.</x:v>
+        <x:v>기록에 나온 정보를 분류 기준과 대조하세요.</x:v>
       </x:c>
       <x:c r="J11" s="9" t="str">
-        <x:v>메모를 누른 뒤 분류함을 누르세요.</x:v>
+        <x:v>상자를 누르고 놓을 곳을 누른 뒤 장치를 작동하세요.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="78.75" customHeight="1">
@@ -706,22 +706,22 @@
         <x:v>이제 네가 가면 돼</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>네 관찰과 모두 맞는 기록 한 장을 고르세요.</x:v>
+        <x:v>네 기록과 맞는 봉투를 찾아 인수함을 여세요.</x:v>
       </x:c>
       <x:c r="F12" s="9" t="str">
         <x:v>친구에게 서로 다른 관찰 결과를 물어보세요.</x:v>
       </x:c>
       <x:c r="G12" s="9" t="str">
-        <x:v>기록 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 기록도 남습니다.</x:v>
+        <x:v>인수 봉투 바만 네 관찰을 함께 만족합니다. 각 관찰을 빼면 해당 특징만 다른 인수 봉투도 남습니다.</x:v>
       </x:c>
       <x:c r="H12" s="9" t="str">
-        <x:v>색·모양·줄 수·재질의 관찰을 모으세요.</x:v>
+        <x:v>장치의 쪽지와 덮개를 눌러 각자 기록을 찾아보세요.</x:v>
       </x:c>
       <x:c r="I12" s="9" t="str">
-        <x:v>조건이 다른 기록을 하나씩 비교하세요.</x:v>
+        <x:v>네 관찰에 모두 맞는 물건인지 비교하세요.</x:v>
       </x:c>
       <x:c r="J12" s="9" t="str">
-        <x:v>마지막 기록을 누르고 정답 확인을 누르세요.</x:v>
+        <x:v>물건을 선택한 뒤 아래 손잡이 버튼을 누르세요.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -801,9 +801,7 @@
       <x:c r="C5" s="9" t="str">
         <x:v>메모 가</x:v>
       </x:c>
-      <x:c r="D5" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D5" s="9" t="str"/>
       <x:c r="E5" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -826,9 +824,7 @@
       <x:c r="C6" s="9" t="str">
         <x:v>메모 나</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D6" s="9" t="str"/>
       <x:c r="E6" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -851,9 +847,7 @@
       <x:c r="C7" s="9" t="str">
         <x:v>메모 다</x:v>
       </x:c>
-      <x:c r="D7" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D7" s="9" t="str"/>
       <x:c r="E7" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -876,9 +870,7 @@
       <x:c r="C8" s="9" t="str">
         <x:v>메모 라</x:v>
       </x:c>
-      <x:c r="D8" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+      <x:c r="D8" s="9" t="str"/>
       <x:c r="E8" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -899,7 +891,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C9" s="9" t="str">
-        <x:v>기록 가</x:v>
+        <x:v>책 가</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
         <x:v>빨강 · 원 · 두 줄 · 종이</x:v>
@@ -924,7 +916,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>기록 나</x:v>
+        <x:v>책 나</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
         <x:v>파랑 · 세모 · 두 줄 · 종이</x:v>
@@ -949,7 +941,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>기록 다</x:v>
+        <x:v>책 다</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
         <x:v>파랑 · 원 · 네 줄 · 종이</x:v>
@@ -974,7 +966,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C12" s="9" t="str">
-        <x:v>기록 라</x:v>
+        <x:v>책 라</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
         <x:v>파랑 · 원 · 두 줄 · 금속</x:v>
@@ -999,7 +991,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C13" s="9" t="str">
-        <x:v>기록 마</x:v>
+        <x:v>책 마</x:v>
       </x:c>
       <x:c r="D13" s="9" t="str">
         <x:v>빨강 · 세모 · 네 줄 · 금속</x:v>
@@ -1024,7 +1016,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>기록 바</x:v>
+        <x:v>책 바</x:v>
       </x:c>
       <x:c r="D14" s="9" t="str">
         <x:v>파랑 · 원 · 두 줄 · 종이</x:v>
@@ -1141,11 +1133,9 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>메모 가</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>기록표 가</x:v>
+      </x:c>
+      <x:c r="D19" s="9" t="str"/>
       <x:c r="E19" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1166,11 +1156,9 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>메모 나</x:v>
-      </x:c>
-      <x:c r="D20" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>기록표 나</x:v>
+      </x:c>
+      <x:c r="D20" s="9" t="str"/>
       <x:c r="E20" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1191,11 +1179,9 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C21" s="9" t="str">
-        <x:v>메모 다</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>기록표 다</x:v>
+      </x:c>
+      <x:c r="D21" s="9" t="str"/>
       <x:c r="E21" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1216,11 +1202,9 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C22" s="9" t="str">
-        <x:v>메모 라</x:v>
-      </x:c>
-      <x:c r="D22" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>기록표 라</x:v>
+      </x:c>
+      <x:c r="D22" s="9" t="str"/>
       <x:c r="E22" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1241,7 +1225,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C23" s="9" t="str">
-        <x:v>기록 가</x:v>
+        <x:v>반납함 가</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
         <x:v>노랑 · 별 · 한 줄 · 금속</x:v>
@@ -1266,7 +1250,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C24" s="9" t="str">
-        <x:v>기록 나</x:v>
+        <x:v>반납함 나</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
         <x:v>빨강 · 세모 · 네 줄 · 금속</x:v>
@@ -1291,7 +1275,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C25" s="9" t="str">
-        <x:v>기록 다</x:v>
+        <x:v>반납함 다</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
         <x:v>노랑 · 별 · 한 줄 · 천</x:v>
@@ -1316,7 +1300,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C26" s="9" t="str">
-        <x:v>기록 라</x:v>
+        <x:v>반납함 라</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
         <x:v>빨강 · 별 · 한 줄 · 천</x:v>
@@ -1341,7 +1325,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C27" s="9" t="str">
-        <x:v>기록 마</x:v>
+        <x:v>반납함 마</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
         <x:v>노랑 · 세모 · 한 줄 · 천</x:v>
@@ -1366,7 +1350,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C28" s="9" t="str">
-        <x:v>기록 바</x:v>
+        <x:v>반납함 바</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
         <x:v>노랑 · 별 · 네 줄 · 천</x:v>
@@ -1391,7 +1375,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>봉투 가</x:v>
+        <x:v>연결표 가</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str"/>
       <x:c r="E29" s="4" t="n">
@@ -1414,7 +1398,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>봉투 나</x:v>
+        <x:v>연결표 나</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str"/>
       <x:c r="E30" s="4" t="n">
@@ -1437,7 +1421,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>봉투 다</x:v>
+        <x:v>연결표 다</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str"/>
       <x:c r="E31" s="4" t="n">
@@ -1460,7 +1444,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>봉투 라</x:v>
+        <x:v>연결표 라</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str"/>
       <x:c r="E32" s="4" t="n">
@@ -1483,11 +1467,9 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C33" s="9" t="str">
-        <x:v>메모 가</x:v>
-      </x:c>
-      <x:c r="D33" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>상자 가</x:v>
+      </x:c>
+      <x:c r="D33" s="9" t="str"/>
       <x:c r="E33" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1508,11 +1490,9 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C34" s="9" t="str">
-        <x:v>메모 나</x:v>
-      </x:c>
-      <x:c r="D34" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>상자 나</x:v>
+      </x:c>
+      <x:c r="D34" s="9" t="str"/>
       <x:c r="E34" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1533,11 +1513,9 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C35" s="9" t="str">
-        <x:v>메모 다</x:v>
-      </x:c>
-      <x:c r="D35" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>상자 다</x:v>
+      </x:c>
+      <x:c r="D35" s="9" t="str"/>
       <x:c r="E35" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1558,11 +1536,9 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C36" s="9" t="str">
-        <x:v>메모 라</x:v>
-      </x:c>
-      <x:c r="D36" s="9" t="str">
-        <x:v>담당자의 단서와 연결</x:v>
-      </x:c>
+        <x:v>상자 라</x:v>
+      </x:c>
+      <x:c r="D36" s="9" t="str"/>
       <x:c r="E36" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
@@ -1583,7 +1559,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="C37" s="9" t="str">
-        <x:v>기록 가</x:v>
+        <x:v>인수 봉투 가</x:v>
       </x:c>
       <x:c r="D37" s="9" t="str">
         <x:v>빨강 · 네모 · 세 줄 · 나무</x:v>
@@ -1608,7 +1584,7 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="C38" s="9" t="str">
-        <x:v>기록 나</x:v>
+        <x:v>인수 봉투 나</x:v>
       </x:c>
       <x:c r="D38" s="9" t="str">
         <x:v>초록 · 세모 · 세 줄 · 나무</x:v>
@@ -1633,7 +1609,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C39" s="9" t="str">
-        <x:v>기록 다</x:v>
+        <x:v>인수 봉투 다</x:v>
       </x:c>
       <x:c r="D39" s="9" t="str">
         <x:v>초록 · 네모 · 네 줄 · 나무</x:v>
@@ -1658,7 +1634,7 @@
         <x:v>D</x:v>
       </x:c>
       <x:c r="C40" s="9" t="str">
-        <x:v>기록 라</x:v>
+        <x:v>인수 봉투 라</x:v>
       </x:c>
       <x:c r="D40" s="9" t="str">
         <x:v>초록 · 네모 · 세 줄 · 금속</x:v>
@@ -1683,7 +1659,7 @@
         <x:v>E</x:v>
       </x:c>
       <x:c r="C41" s="9" t="str">
-        <x:v>기록 마</x:v>
+        <x:v>인수 봉투 마</x:v>
       </x:c>
       <x:c r="D41" s="9" t="str">
         <x:v>빨강 · 세모 · 네 줄 · 금속</x:v>
@@ -1708,7 +1684,7 @@
         <x:v>F</x:v>
       </x:c>
       <x:c r="C42" s="9" t="str">
-        <x:v>기록 바</x:v>
+        <x:v>인수 봉투 바</x:v>
       </x:c>
       <x:c r="D42" s="9" t="str">
         <x:v>초록 · 네모 · 세 줄 · 나무</x:v>
@@ -1974,7 +1950,7 @@
         <x:v>색 관찰</x:v>
       </x:c>
       <x:c r="D9" s="9" t="str">
-        <x:v>내 사진에서 확인한 색: 파랑</x:v>
+        <x:v>내 관찰 책의 색: 파랑</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
         <x:v>B|C|D|F</x:v>
@@ -1991,7 +1967,7 @@
         <x:v>모양 관찰</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>내 사진에서 확인한 모양: 원</x:v>
+        <x:v>내 관찰 책의 모양: 원</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>A|C|D|F</x:v>
@@ -2008,7 +1984,7 @@
         <x:v>줄 관찰</x:v>
       </x:c>
       <x:c r="D11" s="9" t="str">
-        <x:v>내 사진에서 확인한 줄 수: 두 줄</x:v>
+        <x:v>내 관찰 책의 줄 수: 두 줄</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
         <x:v>A|B|D|F</x:v>
@@ -2025,7 +2001,7 @@
         <x:v>재질 관찰</x:v>
       </x:c>
       <x:c r="D12" s="9" t="str">
-        <x:v>내 사진에서 확인한 재질: 종이</x:v>
+        <x:v>내 관찰 책의 재질: 종이</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
         <x:v>A|B|C|F</x:v>
@@ -2107,10 +2083,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C17" s="9" t="str">
-        <x:v>메모 가의 정보</x:v>
+        <x:v>기록표 가의 정보</x:v>
       </x:c>
       <x:c r="D17" s="9" t="str">
-        <x:v>메모 가에 적힌 수: −3</x:v>
+        <x:v>기록표 가에 적힌 수: −3</x:v>
       </x:c>
       <x:c r="E17" s="9" t="str">
         <x:v>A=T2</x:v>
@@ -2124,10 +2100,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C18" s="9" t="str">
-        <x:v>메모 나의 정보</x:v>
+        <x:v>기록표 나의 정보</x:v>
       </x:c>
       <x:c r="D18" s="9" t="str">
-        <x:v>메모 나에 적힌 수: +7</x:v>
+        <x:v>기록표 나에 적힌 수: +7</x:v>
       </x:c>
       <x:c r="E18" s="9" t="str">
         <x:v>B=T1</x:v>
@@ -2141,10 +2117,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C19" s="9" t="str">
-        <x:v>메모 다의 정보</x:v>
+        <x:v>기록표 다의 정보</x:v>
       </x:c>
       <x:c r="D19" s="9" t="str">
-        <x:v>메모 다에 적힌 수: −8</x:v>
+        <x:v>기록표 다에 적힌 수: −8</x:v>
       </x:c>
       <x:c r="E19" s="9" t="str">
         <x:v>C=T2</x:v>
@@ -2158,10 +2134,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C20" s="9" t="str">
-        <x:v>메모 라의 정보</x:v>
+        <x:v>기록표 라의 정보</x:v>
       </x:c>
       <x:c r="D20" s="9" t="str">
-        <x:v>메모 라에 적힌 수: +2</x:v>
+        <x:v>기록표 라에 적힌 수: +2</x:v>
       </x:c>
       <x:c r="E20" s="9" t="str">
         <x:v>D=T1</x:v>
@@ -2178,7 +2154,7 @@
         <x:v>색 관찰</x:v>
       </x:c>
       <x:c r="D21" s="9" t="str">
-        <x:v>내 사진에서 확인한 색: 노랑</x:v>
+        <x:v>내 관찰 반납함의 색: 노랑</x:v>
       </x:c>
       <x:c r="E21" s="9" t="str">
         <x:v>A|C|E|F</x:v>
@@ -2195,7 +2171,7 @@
         <x:v>모양 관찰</x:v>
       </x:c>
       <x:c r="D22" s="9" t="str">
-        <x:v>내 사진에서 확인한 모양: 별</x:v>
+        <x:v>내 관찰 반납함의 모양: 별</x:v>
       </x:c>
       <x:c r="E22" s="9" t="str">
         <x:v>A|C|D|F</x:v>
@@ -2212,7 +2188,7 @@
         <x:v>줄 관찰</x:v>
       </x:c>
       <x:c r="D23" s="9" t="str">
-        <x:v>내 사진에서 확인한 줄 수: 한 줄</x:v>
+        <x:v>내 관찰 반납함의 줄 수: 한 줄</x:v>
       </x:c>
       <x:c r="E23" s="9" t="str">
         <x:v>A|C|D|E</x:v>
@@ -2229,7 +2205,7 @@
         <x:v>재질 관찰</x:v>
       </x:c>
       <x:c r="D24" s="9" t="str">
-        <x:v>내 사진에서 확인한 재질: 천</x:v>
+        <x:v>내 관찰 반납함의 재질: 천</x:v>
       </x:c>
       <x:c r="E24" s="9" t="str">
         <x:v>C|D|E|F</x:v>
@@ -2246,7 +2222,7 @@
         <x:v>앞뒤 메모</x:v>
       </x:c>
       <x:c r="D25" s="9" t="str">
-        <x:v>가 봉투는 나 봉투보다 뒤에 놓는다.</x:v>
+        <x:v>가 연결표는 나 연결표보다 뒤에 놓는다.</x:v>
       </x:c>
       <x:c r="E25" s="9" t="str">
         <x:v>A&gt;B</x:v>
@@ -2263,7 +2239,7 @@
         <x:v>간격 메모</x:v>
       </x:c>
       <x:c r="D26" s="9" t="str">
-        <x:v>가 봉투와 나 봉투는 붙여 놓지 않는다.</x:v>
+        <x:v>가 연결표와 나 연결표는 붙여 놓지 않는다.</x:v>
       </x:c>
       <x:c r="E26" s="9" t="str">
         <x:v>A!~B</x:v>
@@ -2280,7 +2256,7 @@
         <x:v>전달 메모</x:v>
       </x:c>
       <x:c r="D27" s="9" t="str">
-        <x:v>가 봉투는 라 봉투보다 뒤에 놓는다.</x:v>
+        <x:v>가 연결표는 라 연결표보다 뒤에 놓는다.</x:v>
       </x:c>
       <x:c r="E27" s="9" t="str">
         <x:v>A&gt;D</x:v>
@@ -2297,7 +2273,7 @@
         <x:v>끝자리 메모</x:v>
       </x:c>
       <x:c r="D28" s="9" t="str">
-        <x:v>가 봉투는 마지막에 놓지 않는다.</x:v>
+        <x:v>가 연결표는 마지막에 놓지 않는다.</x:v>
       </x:c>
       <x:c r="E28" s="9" t="str">
         <x:v>A!=4</x:v>
@@ -2311,10 +2287,10 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="C29" s="9" t="str">
-        <x:v>메모 가의 정보</x:v>
+        <x:v>상자 가의 정보</x:v>
       </x:c>
       <x:c r="D29" s="9" t="str">
-        <x:v>메모 가에 적힌 생물: 고양이</x:v>
+        <x:v>상자 가에 적힌 생물: 고양이</x:v>
       </x:c>
       <x:c r="E29" s="9" t="str">
         <x:v>A=T1</x:v>
@@ -2328,10 +2304,10 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C30" s="9" t="str">
-        <x:v>메모 나의 정보</x:v>
+        <x:v>상자 나의 정보</x:v>
       </x:c>
       <x:c r="D30" s="9" t="str">
-        <x:v>메모 나에 적힌 생물: 장미</x:v>
+        <x:v>상자 나에 적힌 생물: 장미</x:v>
       </x:c>
       <x:c r="E30" s="9" t="str">
         <x:v>B=T2</x:v>
@@ -2345,10 +2321,10 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="C31" s="9" t="str">
-        <x:v>메모 다의 정보</x:v>
+        <x:v>상자 다의 정보</x:v>
       </x:c>
       <x:c r="D31" s="9" t="str">
-        <x:v>메모 다에 적힌 생물: 민들레</x:v>
+        <x:v>상자 다에 적힌 생물: 민들레</x:v>
       </x:c>
       <x:c r="E31" s="9" t="str">
         <x:v>C=T2</x:v>
@@ -2362,10 +2338,10 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="C32" s="9" t="str">
-        <x:v>메모 라의 정보</x:v>
+        <x:v>상자 라의 정보</x:v>
       </x:c>
       <x:c r="D32" s="9" t="str">
-        <x:v>메모 라에 적힌 생물: 강아지</x:v>
+        <x:v>상자 라에 적힌 생물: 강아지</x:v>
       </x:c>
       <x:c r="E32" s="9" t="str">
         <x:v>D=T1</x:v>
@@ -2382,7 +2358,7 @@
         <x:v>색 관찰</x:v>
       </x:c>
       <x:c r="D33" s="9" t="str">
-        <x:v>내 사진에서 확인한 색: 초록</x:v>
+        <x:v>내 관찰 인수 봉투의 색: 초록</x:v>
       </x:c>
       <x:c r="E33" s="9" t="str">
         <x:v>B|C|D|F</x:v>
@@ -2399,7 +2375,7 @@
         <x:v>모양 관찰</x:v>
       </x:c>
       <x:c r="D34" s="9" t="str">
-        <x:v>내 사진에서 확인한 모양: 네모</x:v>
+        <x:v>내 관찰 인수 봉투의 모양: 네모</x:v>
       </x:c>
       <x:c r="E34" s="9" t="str">
         <x:v>A|C|D|F</x:v>
@@ -2416,7 +2392,7 @@
         <x:v>줄 관찰</x:v>
       </x:c>
       <x:c r="D35" s="9" t="str">
-        <x:v>내 사진에서 확인한 줄 수: 세 줄</x:v>
+        <x:v>내 관찰 인수 봉투의 줄 수: 세 줄</x:v>
       </x:c>
       <x:c r="E35" s="9" t="str">
         <x:v>A|B|D|F</x:v>
@@ -2433,7 +2409,7 @@
         <x:v>재질 관찰</x:v>
       </x:c>
       <x:c r="D36" s="9" t="str">
-        <x:v>내 사진에서 확인한 재질: 나무</x:v>
+        <x:v>내 관찰 인수 봉투의 재질: 나무</x:v>
       </x:c>
       <x:c r="E36" s="9" t="str">
         <x:v>A|B|C|F</x:v>

</xml_diff>